<commit_message>
#2 peripheral Module link update
</commit_message>
<xml_diff>
--- a/Design-Files/Deliverables/BOM/eSpark BOM.xlsx
+++ b/Design-Files/Deliverables/BOM/eSpark BOM.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="570" uniqueCount="335">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="570" uniqueCount="334">
   <si>
     <t>Component list</t>
   </si>
@@ -1021,9 +1021,6 @@
   </si>
   <si>
     <t>High sensitivity wireless remote control receiving module RXB61 multiple frequency 315M.433MHZ</t>
-  </si>
-  <si>
-    <t>Alibaba</t>
   </si>
 </sst>
 </file>
@@ -1031,9 +1028,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="3">
-    <numFmt numFmtId="166" formatCode="[$-409]h:mm:ss\ AM/PM;@"/>
-    <numFmt numFmtId="167" formatCode="&quot;$&quot;#,##0.0000"/>
-    <numFmt numFmtId="168" formatCode="&quot;$&quot;#,##0.00"/>
+    <numFmt numFmtId="164" formatCode="[$-409]h:mm:ss\ AM/PM;@"/>
+    <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.0000"/>
+    <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
   <fonts count="25">
     <font>
@@ -1542,7 +1539,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="166" fontId="9" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="9" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1614,16 +1611,16 @@
     <xf numFmtId="0" fontId="21" fillId="2" borderId="10" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="17" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="17" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="2" borderId="11" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="17" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="17" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="18" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="18" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1635,10 +1632,10 @@
     <xf numFmtId="0" fontId="18" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="168" fontId="4" fillId="3" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="4" fillId="3" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="168" fontId="4" fillId="3" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="4" fillId="3" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -5278,17 +5275,17 @@
         <v>5</v>
       </c>
       <c r="N63" s="34">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="O63" s="51" t="s">
-        <v>334</v>
+        <v>282</v>
       </c>
       <c r="P63" s="52">
-        <v>2.6</v>
+        <v>2</v>
       </c>
       <c r="Q63" s="52">
         <f t="shared" si="5"/>
-        <v>15.600000000000001</v>
+        <v>10</v>
       </c>
       <c r="R63" s="34"/>
       <c r="S63" s="57"/>
@@ -5314,7 +5311,7 @@
       <c r="P64" s="67"/>
       <c r="Q64" s="59">
         <f>SUM(Q10:Q63)</f>
-        <v>137.16720000000001</v>
+        <v>131.56720000000001</v>
       </c>
       <c r="R64" s="70"/>
       <c r="S64" s="71"/>
@@ -5340,7 +5337,7 @@
       <c r="P65" s="67"/>
       <c r="Q65" s="60">
         <f>Q64/5</f>
-        <v>27.433440000000001</v>
+        <v>26.313440000000003</v>
       </c>
       <c r="R65" s="72"/>
       <c r="S65" s="73"/>

</xml_diff>